<commit_message>
powiekszenie grupowania do 2 wyników
</commit_message>
<xml_diff>
--- a/grupowane.xlsx
+++ b/grupowane.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -485,19 +485,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>6.6</v>
+        <v>3.1</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>G</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>F60</t>
+          <t>G87</t>
         </is>
       </c>
     </row>
@@ -508,19 +508,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>6.9</v>
+        <v>6.6</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>G100</t>
+          <t>F60</t>
         </is>
       </c>
     </row>
@@ -531,19 +531,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C5" t="n">
-        <v>8.699999999999999</v>
+        <v>4.8</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>G3</t>
+          <t>G</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>F48</t>
+          <t>F60</t>
         </is>
       </c>
     </row>
@@ -554,33 +554,33 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C6" t="n">
-        <v>5.8</v>
+        <v>6.9</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>G</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>F48</t>
+          <t>G100</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>baksztag</t>
+          <t>bajdewind</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C7" t="n">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -589,76 +589,76 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>F60</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>baksztag</t>
+          <t>bajdewind</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C8" t="n">
-        <v>5.9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>G3</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>F60</t>
+          <t>F48</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>baksztag</t>
+          <t>bajdewind</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C9" t="n">
-        <v>8.9</v>
+        <v>6.6</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>G100</t>
+          <t>F60</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>baksztag</t>
+          <t>bajdewind</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C10" t="n">
-        <v>10</v>
+        <v>5.8</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>F60</t>
+          <t>F48</t>
         </is>
       </c>
     </row>
@@ -669,10 +669,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C11" t="n">
-        <v>9.4</v>
+        <v>7</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -681,7 +681,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">G87 </t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -692,10 +692,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C12" t="n">
-        <v>9.6</v>
+        <v>3.7</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -704,7 +704,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>G87</t>
+          <t>S</t>
         </is>
       </c>
     </row>
@@ -715,10 +715,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C13" t="n">
-        <v>9.800000000000001</v>
+        <v>5.9</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -734,14 +734,14 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>fordewind</t>
+          <t>baksztag</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C14" t="n">
-        <v>3.6</v>
+        <v>5.6</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -750,21 +750,21 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>F60</t>
+          <t>G87</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>fordewind</t>
+          <t>baksztag</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C15" t="n">
-        <v>8.1</v>
+        <v>8.9</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -773,25 +773,25 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>G100</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>fordewind</t>
+          <t>baksztag</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>3</v>
       </c>
       <c r="C16" t="n">
-        <v>6.2</v>
+        <v>7.6</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>G</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -803,14 +803,14 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>fordewind</t>
+          <t>baksztag</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>4</v>
       </c>
       <c r="C17" t="n">
-        <v>6.1</v>
+        <v>10</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -819,21 +819,21 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>G100</t>
+          <t>F60</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>fordewind</t>
+          <t>baksztag</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>8.5</v>
+        <v>9.5</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -842,21 +842,21 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>G87</t>
+          <t>S</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>fordewind</t>
+          <t>baksztag</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>8.5</v>
+        <v>9.4</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -865,21 +865,21 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>S</t>
+          <t xml:space="preserve">G87 </t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ostry bajdewind</t>
+          <t>baksztag</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>3.6</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -888,21 +888,21 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>F60</t>
+          <t>G87</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ostry bajdewind</t>
+          <t>baksztag</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C21" t="n">
-        <v>4.6</v>
+        <v>9.6</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -911,21 +911,21 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>F60</t>
+          <t>G87</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ostry bajdewind</t>
+          <t>baksztag</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C22" t="n">
-        <v>5</v>
+        <v>9.6</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -941,14 +941,14 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ostry bajdewind</t>
+          <t>baksztag</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C23" t="n">
-        <v>6.1</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -957,44 +957,44 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>G100</t>
+          <t>F60</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ostry baksztag</t>
+          <t>baksztag</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C24" t="n">
-        <v>1.9</v>
+        <v>7.3</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>F60</t>
+          <t>F48</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ostry baksztag</t>
+          <t>fordewind</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C25" t="n">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1010,14 +1010,14 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ostry baksztag</t>
+          <t>fordewind</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C26" t="n">
-        <v>6.6</v>
+        <v>1.1</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1033,14 +1033,14 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ostry baksztag</t>
+          <t>fordewind</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>10</v>
+        <v>8.1</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1049,90 +1049,90 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>G87</t>
+          <t>S</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ostry baksztag</t>
+          <t>fordewind</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C28" t="n">
-        <v>10.3</v>
+        <v>6.5</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>G87</t>
+          <t>F60</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ostry baksztag</t>
+          <t>fordewind</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C29" t="n">
-        <v>9</v>
+        <v>6.2</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>G2</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>F48</t>
+          <t>F60</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ostry baksztag</t>
+          <t>fordewind</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C30" t="n">
-        <v>8.6</v>
+        <v>5.8</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>G2</t>
+          <t>G</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>F30</t>
+          <t>S</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>pelny bajdewind</t>
+          <t>fordewind</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C31" t="n">
-        <v>5.5</v>
+        <v>6.1</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1141,25 +1141,25 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>F60</t>
+          <t>G100</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>pelny bajdewind</t>
+          <t>fordewind</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C32" t="n">
-        <v>7.3</v>
+        <v>4.8</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1171,14 +1171,14 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>pelny bajdewind</t>
+          <t>fordewind</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C33" t="n">
-        <v>8.9</v>
+        <v>8.5</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1194,37 +1194,37 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>pelny bajdewind</t>
+          <t>fordewind</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>5</v>
       </c>
       <c r="C34" t="n">
-        <v>9.699999999999999</v>
+        <v>5.1</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>G100</t>
+          <t>F48</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>pelny bajdewind</t>
+          <t>fordewind</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>6</v>
       </c>
       <c r="C35" t="n">
-        <v>8.199999999999999</v>
+        <v>8.5</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1233,21 +1233,21 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>G100</t>
+          <t>S</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>pelny baksztag</t>
+          <t>fordewind</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C36" t="n">
-        <v>8.5</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1263,18 +1263,18 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>pelny baksztag</t>
+          <t>ostry bajdewind</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C37" t="n">
-        <v>7.8</v>
+        <v>3.6</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>G2</t>
+          <t>G</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1286,14 +1286,14 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>pelny baksztag</t>
+          <t>ostry bajdewind</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C38" t="n">
-        <v>8.300000000000001</v>
+        <v>4.6</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1302,22 +1302,22 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>F60</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>pelny baksztag</t>
+          <t>ostry bajdewind</t>
         </is>
       </c>
       <c r="B39" t="n">
+        <v>4</v>
+      </c>
+      <c r="C39" t="n">
         <v>5</v>
       </c>
-      <c r="C39" t="n">
-        <v>10.2</v>
-      </c>
       <c r="D39" t="inlineStr">
         <is>
           <t>G</t>
@@ -1325,21 +1325,21 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>G87</t>
+          <t>F60</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>polwiatr</t>
+          <t>ostry bajdewind</t>
         </is>
       </c>
       <c r="B40" t="n">
+        <v>4</v>
+      </c>
+      <c r="C40" t="n">
         <v>2</v>
-      </c>
-      <c r="C40" t="n">
-        <v>2.9</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1355,14 +1355,14 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>polwiatr</t>
+          <t>ostry bajdewind</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C41" t="n">
-        <v>8</v>
+        <v>6.1</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -1378,67 +1378,941 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>polwiatr</t>
+          <t>ostry bajdewind</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C42" t="n">
-        <v>7.9</v>
+        <v>4.7</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>G3</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>G100</t>
+          <t>F48</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>polwiatr</t>
+          <t>ostry baksztag</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C43" t="n">
-        <v>9.5</v>
+        <v>1.9</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>G3</t>
+          <t>G</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>F48</t>
+          <t>F60</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>ostry baksztag</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>2</v>
+      </c>
+      <c r="C44" t="n">
+        <v>4</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>F60</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ostry baksztag</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>2</v>
+      </c>
+      <c r="C45" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>F60</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ostry baksztag</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>3</v>
+      </c>
+      <c r="C46" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>F60</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>ostry baksztag</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>3</v>
+      </c>
+      <c r="C47" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>F60</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>ostry baksztag</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>4</v>
+      </c>
+      <c r="C48" t="n">
+        <v>10</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>G87</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>ostry baksztag</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>4</v>
+      </c>
+      <c r="C49" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>G87</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>ostry baksztag</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>5</v>
+      </c>
+      <c r="C50" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>G87</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>ostry baksztag</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>5</v>
+      </c>
+      <c r="C51" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>G87</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ostry baksztag</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>6</v>
+      </c>
+      <c r="C52" t="n">
+        <v>9</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>G2</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>F48</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>ostry baksztag</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>6</v>
+      </c>
+      <c r="C53" t="n">
+        <v>9</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>F60</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ostry baksztag</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>7</v>
+      </c>
+      <c r="C54" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>G2</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>F30</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>ostry baksztag</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>7</v>
+      </c>
+      <c r="C55" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>G2</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>F30</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>pelny bajdewind</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>2</v>
+      </c>
+      <c r="C56" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>F60</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>pelny bajdewind</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>2</v>
+      </c>
+      <c r="C57" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>F60</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>pelny bajdewind</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>3</v>
+      </c>
+      <c r="C58" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>F60</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>pelny bajdewind</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>3</v>
+      </c>
+      <c r="C59" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>G100</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>pelny bajdewind</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>4</v>
+      </c>
+      <c r="C60" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>G87</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>pelny bajdewind</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>4</v>
+      </c>
+      <c r="C61" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>G87</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>pelny bajdewind</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>5</v>
+      </c>
+      <c r="C62" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>G100</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>pelny bajdewind</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>5</v>
+      </c>
+      <c r="C63" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>G100</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>pelny bajdewind</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>6</v>
+      </c>
+      <c r="C64" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>G100</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>pelny baksztag</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>2</v>
+      </c>
+      <c r="C65" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>pelny baksztag</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>2</v>
+      </c>
+      <c r="C66" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>F60</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>pelny baksztag</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>3</v>
+      </c>
+      <c r="C67" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>G2</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>F60</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>pelny baksztag</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>3</v>
+      </c>
+      <c r="C68" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>G2</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>F60</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>pelny baksztag</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>4</v>
+      </c>
+      <c r="C69" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>pelny baksztag</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>4</v>
+      </c>
+      <c r="C70" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>G100</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>pelny baksztag</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>5</v>
+      </c>
+      <c r="C71" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>G87</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>pelny baksztag</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>5</v>
+      </c>
+      <c r="C72" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>F60</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
           <t>polwiatr</t>
         </is>
       </c>
-      <c r="B44" t="n">
+      <c r="B73" t="n">
+        <v>2</v>
+      </c>
+      <c r="C73" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>F60</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>polwiatr</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>2</v>
+      </c>
+      <c r="C74" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>F60</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>polwiatr</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>3</v>
+      </c>
+      <c r="C75" t="n">
+        <v>8</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>G100</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>polwiatr</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>3</v>
+      </c>
+      <c r="C76" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>F60</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>polwiatr</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>4</v>
+      </c>
+      <c r="C77" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>G100</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>polwiatr</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>4</v>
+      </c>
+      <c r="C78" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>G100</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>polwiatr</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>5</v>
+      </c>
+      <c r="C79" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>F48</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>polwiatr</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>5</v>
+      </c>
+      <c r="C80" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>G87</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>polwiatr</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
         <v>6</v>
       </c>
-      <c r="C44" t="n">
+      <c r="C81" t="n">
         <v>8.4</v>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D81" t="inlineStr">
         <is>
           <t>G1</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>G100</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>polwiatr</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>6</v>
+      </c>
+      <c r="C82" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
         <is>
           <t>G100</t>
         </is>

</xml_diff>

<commit_message>
rodzielenie dziennika na 2 czesci
</commit_message>
<xml_diff>
--- a/grupowane.xlsx
+++ b/grupowane.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>